<commit_message>
gantt: operadores Bimbo validados
</commit_message>
<xml_diff>
--- a/gantt-piloto-2026-10-29.xlsx
+++ b/gantt-piloto-2026-10-29.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="355">
   <si>
     <t xml:space="preserve">Grupo Bimbo × Uvicuo · Plan de arranque del piloto de peajes</t>
   </si>
@@ -635,7 +635,7 @@
     <t xml:space="preserve">Validación de la lista · Bimbo</t>
   </si>
   <si>
-    <t xml:space="preserve">La operación de Bimbo Sureste confirma qué operadores y qué unidades de la lista entran al piloto.</t>
+    <t xml:space="preserve">Giselle (Bimbo Sureste) validó y devolvió las listas: operadores de Región Sur (161, con sus altas marcadas) y unidades RS con su centro/ubicación.</t>
   </si>
   <si>
     <t xml:space="preserve">Cada jefe de transporte revisa al tener acceso a la plataforma</t>
@@ -7632,7 +7632,7 @@
         <v>76</v>
       </c>
       <c r="I45" s="22" t="s">
-        <v>90</v>
+        <v>32</v>
       </c>
       <c r="J45" s="19"/>
       <c r="K45" s="15" t="s">
@@ -7643,11 +7643,11 @@
         <v>46317</v>
       </c>
       <c r="M45" s="24" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="N45" s="23"/>
       <c r="O45" s="23" t="n">
-        <v>46319</v>
+        <v>46324</v>
       </c>
       <c r="P45" s="22" t="s">
         <v>34</v>
@@ -7741,9 +7741,7 @@
       <c r="I46" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="J46" s="34" t="s">
-        <v>76</v>
-      </c>
+      <c r="J46" s="19"/>
       <c r="K46" s="15" t="s">
         <v>100</v>
       </c>
@@ -7849,9 +7847,7 @@
       <c r="I47" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="J47" s="34" t="s">
-        <v>76</v>
-      </c>
+      <c r="J47" s="19"/>
       <c r="K47" s="15" t="s">
         <v>100</v>
       </c>

</xml_diff>